<commit_message>
bugs fixed, some examples added
</commit_message>
<xml_diff>
--- a/examples/ex070.MF_Separator.xlsx
+++ b/examples/ex070.MF_Separator.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ЭтаКнига" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\unifloc\unifloc_vba\examples\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\unifloc\unifloc_vba\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE95C267-D2F3-4D6C-B391-208EF6499D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27C87DD6-BEF1-416C-B46F-1C94358EE37A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{E2E84BD7-C2A2-4E24-A35E-70B40629F858}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21390" xr2:uid="{E2E84BD7-C2A2-4E24-A35E-70B40629F858}"/>
   </bookViews>
   <sheets>
     <sheet name="Общая сепарация на скважине" sheetId="2" r:id="rId1"/>
@@ -632,8 +632,30 @@
 </comments>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="62">
   <si>
     <t>gamma_gas</t>
   </si>
@@ -807,6 +829,18 @@
   </si>
   <si>
     <t>well_ksep_full_d</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>gas fraction feed</t>
+  </si>
+  <si>
+    <t>gas fraction in pump</t>
+  </si>
+  <si>
+    <t>gas fraction in gs</t>
   </si>
 </sst>
 </file>
@@ -1088,67 +1122,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>0.996</c:v>
+                  <c:v>0.997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.97199999999999998</c:v>
+                  <c:v>0.97299999999999998</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.93899999999999995</c:v>
+                  <c:v>0.94099999999999995</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.9</c:v>
+                  <c:v>0.90200000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.86199999999999999</c:v>
+                  <c:v>0.86499999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.81399999999999995</c:v>
+                  <c:v>0.81699999999999995</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.70299999999999996</c:v>
+                  <c:v>0.73599999999999999</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.52600000000000002</c:v>
+                  <c:v>0.629</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.35</c:v>
+                  <c:v>0.53100000000000003</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.193</c:v>
+                  <c:v>0.45100000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.9E-2</c:v>
+                  <c:v>0.39200000000000002</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6999999999999998E-2</c:v>
+                  <c:v>0.373</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.5999999999999997E-2</c:v>
+                  <c:v>0.35599999999999998</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.4000000000000002E-2</c:v>
+                  <c:v>0.34200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.33</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.32</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.311</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.30399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.29799999999999999</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.29199999999999998</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.28799999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1269,67 +1303,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>0.96399999999999997</c:v>
+                  <c:v>0.97299999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.82899999999999996</c:v>
+                  <c:v>0.83699999999999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.73099999999999998</c:v>
+                  <c:v>0.73799999999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.65200000000000002</c:v>
+                  <c:v>0.65900000000000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.60699999999999998</c:v>
+                  <c:v>0.61299999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.55400000000000005</c:v>
+                  <c:v>0.56000000000000005</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.46400000000000002</c:v>
+                  <c:v>0.51500000000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.34899999999999998</c:v>
+                  <c:v>0.47599999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.251</c:v>
+                  <c:v>0.44400000000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.16600000000000001</c:v>
+                  <c:v>0.41599999999999998</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>3.9E-2</c:v>
+                  <c:v>0.39200000000000002</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>3.6999999999999998E-2</c:v>
+                  <c:v>0.373</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>3.5999999999999997E-2</c:v>
+                  <c:v>0.35599999999999998</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>3.4000000000000002E-2</c:v>
+                  <c:v>0.34200000000000003</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.33</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.32</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.311</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.30399999999999999</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.29799999999999999</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.29199999999999998</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>0.28799999999999998</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1453,7 +1487,7 @@
                   <c:v>0.88600000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.83299999999999996</c:v>
+                  <c:v>0.83399999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0.77500000000000002</c:v>
@@ -1462,22 +1496,22 @@
                   <c:v>0.71299999999999997</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.65</c:v>
+                  <c:v>0.65100000000000002</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.58399999999999996</c:v>
+                  <c:v>0.58499999999999996</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.44700000000000001</c:v>
+                  <c:v>0.45500000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.27200000000000002</c:v>
+                  <c:v>0.29099999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.13200000000000001</c:v>
+                  <c:v>0.158</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>3.3000000000000002E-2</c:v>
+                  <c:v>0.06</c:v>
                 </c:pt>
                 <c:pt idx="10">
                   <c:v>0</c:v>
@@ -2034,67 +2068,67 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>66.099999999999994</c:v>
+                  <c:v>66.156000000000006</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>707.33399999999995</c:v>
+                  <c:v>708.28599999999994</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1305.4490000000001</c:v>
+                  <c:v>1307.8050000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1845.4059999999999</c:v>
+                  <c:v>1849.6010000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2336.1129999999998</c:v>
+                  <c:v>2342.6129999999998</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>2740.8629999999998</c:v>
+                  <c:v>2749.76</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>2615.1880000000001</c:v>
+                  <c:v>2747.19</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1527.1949999999999</c:v>
+                  <c:v>2032.7190000000001</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-225.703</c:v>
+                  <c:v>815.03</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>-2479.1370000000002</c:v>
+                  <c:v>-808.11300000000006</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>-5979.63</c:v>
+                  <c:v>-3480.7289999999998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>-6489.3670000000002</c:v>
+                  <c:v>-3973.998</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>-7193.7539999999999</c:v>
+                  <c:v>-4469.0510000000004</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>-7686.0879999999997</c:v>
+                  <c:v>-4963.6130000000003</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>-9428.58</c:v>
+                  <c:v>-6435.6469999999999</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>-10230.709999999999</c:v>
+                  <c:v>-6862.799</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>-10767.948</c:v>
+                  <c:v>-7409.66</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>-11437.579</c:v>
+                  <c:v>-7953.0540000000001</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>-12265.919</c:v>
+                  <c:v>-8493.4290000000001</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>-12944.267</c:v>
+                  <c:v>-9031.607</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>-13622.606</c:v>
+                  <c:v>-9568.7350000000006</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2618,31 +2652,31 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
-                  <c:v>0.23200000000000001</c:v>
+                  <c:v>0.23300000000000001</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>2.2229999999999999</c:v>
+                  <c:v>2.2410000000000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>3.37</c:v>
+                  <c:v>3.4159999999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3.3809999999999998</c:v>
+                  <c:v>3.4630000000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2.4300000000000002</c:v>
+                  <c:v>2.5569999999999999</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-0.20200000000000001</c:v>
+                  <c:v>-2.8000000000000001E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-13.199</c:v>
+                  <c:v>-10.619</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-45.003</c:v>
+                  <c:v>-35.122999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>-131.68600000000001</c:v>
+                  <c:v>-69.463999999999999</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>-167.85499999999999</c:v>
@@ -3053,6 +3087,978 @@
             </a:pPr>
             <a:r>
               <a:rPr lang="en-US"/>
+              <a:t>gas fraction in pump</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Общая сепарация на скважине'!$T$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>gas fraction feed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Общая сепарация на скважине'!$H$10:$H$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>20.9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30.85</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.799999999999997</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.75</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>60.7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>70.650000000000006</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80.599999999999994</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>90.55</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>100.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>110.45</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>120.4</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>130.35</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>140.30000000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>150.25</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>160.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>170.15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>180.1</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>190.05</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Общая сепарация на скважине'!$T$10:$T$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.55350477167797996</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.55350477167797996</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.55350477167798007</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F53C-4AC8-8A27-0664B7A6FE28}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Общая сепарация на скважине'!$U$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>gas fraction in pump</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Общая сепарация на скважине'!$H$10:$H$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>20.9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30.85</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.799999999999997</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.75</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>60.7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>70.650000000000006</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80.599999999999994</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>90.55</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>100.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>110.45</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>120.4</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>130.35</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>140.30000000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>150.25</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>160.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>170.15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>180.1</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>190.05</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Общая сепарация на скважине'!$U$10:$U$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>9.7236563602478912E-3</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.2845064602382593E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>4.1094197807267863E-2</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>6.2777248767335814E-2</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.2885857814671157E-2</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.10732774085061607</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.16843619621973591</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.26179777427701612</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.34511980621007499</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.41273119641773265</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.48442215735325556</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.48771028188520732</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.49044918942208804</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.49272556975681142</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.51076729949079169</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.51016877555079976</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.51140404733152833</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.512508622496747</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.513450629685963</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.51419031206811949</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.51490847339588086</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-F53C-4AC8-8A27-0664B7A6FE28}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'Общая сепарация на скважине'!$V$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>gas fraction in gs</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Общая сепарация на скважине'!$H$10:$H$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>10.95</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>20.9</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>30.85</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>40.799999999999997</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>50.75</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>60.7</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>70.650000000000006</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>80.599999999999994</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>90.55</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>100.5</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>110.45</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>120.4</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>130.35</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>140.30000000000001</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>150.25</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>160.19999999999999</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>170.15</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>180.1</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>190.05</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>200</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Общая сепарация на скважине'!$V$10:$V$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="21"/>
+                <c:pt idx="0">
+                  <c:v>2.5533933853236015E-2</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>9.9050458581768572E-2</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.14583284377950637</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.1794397586713847</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.19772138038641024</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.21797774972556341</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.26653454983912028</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.33024790287712152</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.3819379134772044</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.42503786661386767</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.48442215735325556</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.48771028188520732</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.49044918942208804</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.49272556975681142</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.50860666940773758</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.51016877555079976</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.51140404733152833</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.512508622496747</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>0.513450629685963</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>0.51419031206811949</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>0.51490847339588086</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-F53C-4AC8-8A27-0664B7A6FE28}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1409267775"/>
+        <c:axId val="1409269215"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1409267775"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Qliq, sm3/day</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="ru-RU"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1409269215"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1409269215"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Ksep</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="ru-RU"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="ru-RU"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1409267775"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="ru-RU"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="ru-RU"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="ru-RU"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
               <a:t>gassep curve</a:t>
             </a:r>
           </a:p>
@@ -3208,7 +4214,7 @@
                   <c:v>0.87615094196922993</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.85841925945936737</c:v>
+                  <c:v>0.85841925945936748</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.83587912237352002</c:v>
@@ -3217,10 +4223,10 @@
                   <c:v>0.80853053071168746</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.77637348447386989</c:v>
+                  <c:v>0.77637348447387</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.73940798366006733</c:v>
+                  <c:v>0.73940798366006744</c:v>
                 </c:pt>
                 <c:pt idx="8">
                   <c:v>0.6975761453613416</c:v>
@@ -3599,7 +4605,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="ru-RU"/>
@@ -3810,34 +4816,34 @@
                   <c:v>0.85966072078600009</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.8259751192560002</c:v>
+                  <c:v>0.82597511925599998</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.7775493509260003</c:v>
+                  <c:v>0.77754935092600019</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.71760875854599993</c:v>
+                  <c:v>0.71760875854600004</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.65069857986600033</c:v>
+                  <c:v>0.6506985798660001</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.58268394763599962</c:v>
+                  <c:v>0.58268394763600018</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.52074988960600077</c:v>
+                  <c:v>0.52074988960600022</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.47340132852599986</c:v>
+                  <c:v>0.47340132852600031</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.42574987164024719</c:v>
+                  <c:v>0.42574987164025058</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.33170162999063563</c:v>
+                  <c:v>0.3317016299906379</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.18978500611055324</c:v>
+                  <c:v>0.18978500611055438</c:v>
                 </c:pt>
                 <c:pt idx="20">
                   <c:v>0</c:v>
@@ -4180,7 +5186,7 @@
 </c:chartSpace>
 </file>
 
-<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/charts/chart7.xml><?xml version="1.0" encoding="utf-8"?>
 <c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
   <c:date1904 val="0"/>
   <c:lang val="ru-RU"/>
@@ -5001,6 +6007,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -8097,20 +9143,536 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style7.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>257175</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>180975</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>185056</xdr:rowOff>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>504824</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>171450</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8137,16 +9699,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>249011</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>160564</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>26</xdr:col>
+      <xdr:col>32</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>185056</xdr:rowOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>108857</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8173,16 +9735,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>26</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>608240</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>119743</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>34</xdr:col>
-      <xdr:colOff>1</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>185056</xdr:rowOff>
+      <xdr:col>39</xdr:col>
+      <xdr:colOff>149678</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>122464</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8443,6 +10005,93 @@
     </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>514350</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>180975</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="6" name="Диаграмма 5">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1808BA77-6645-452E-B01E-8834CA657E94}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>212912</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>67235</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>393854</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>33617</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Рисунок 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E17D3D48-11B4-4014-AA9F-6928BC84C9BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="32420" t="9968" r="37389" b="9714"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="212912" y="3877235"/>
+          <a:ext cx="2153177" cy="3395382"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -8527,16 +10176,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>2</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>161925</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>504825</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>185056</xdr:rowOff>
+      <xdr:rowOff>156481</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8582,6 +10231,7 @@
       <definedName name="encode_PVT"/>
       <definedName name="ESP_gassep_ksep_d"/>
       <definedName name="ESP_gassep_name"/>
+      <definedName name="feed_gas_fraction_d"/>
       <definedName name="well_ksep_full_d"/>
       <definedName name="well_ksep_natural_d"/>
     </definedNames>
@@ -8910,14 +10560,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{867DFA60-36E6-4C76-B5E9-D55899FFF512}">
   <sheetPr codeName="Лист1"/>
-  <dimension ref="B3:R41"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="B3:V41"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.4609375" customWidth="1"/>
-    <col min="5" max="5" width="19.3828125" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="5" max="5" width="19.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>0</v>
       </c>
@@ -8936,8 +10586,11 @@
       <c r="I3" s="2">
         <v>50</v>
       </c>
+      <c r="J3" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="4" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -8956,8 +10609,11 @@
       <c r="I4" s="2">
         <v>40</v>
       </c>
+      <c r="J4" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="5" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>2</v>
       </c>
@@ -8977,8 +10633,11 @@
         <f>feed_json_1</f>
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":30,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
+      <c r="J5" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="6" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -8996,10 +10655,13 @@
       </c>
       <c r="I6" s="2" t="str">
         <f>gas_separation_json</f>
-        <v>{"calc_mode":"by_correlation","natsep_model":"0","d_intake_mm":"92","d_cas_mm":"125","d_tub_mm":"72","pkv_period_ratio":"0.5","gassep_type":"0","gassep_qnom_sm3day":"200","param":{"show_array":1,"gas_goes_into_solution":1,"calibr_li":2}}</v>
+        <v>{"calc_mode":"by_correlation","natsep_model":0,"d_intake_mm":92,"d_cas_mm":125,"d_tub_mm":72,"pkv_period_ratio":0.5,"gassep_type":-1,"gassep_qnom_sm3day":200,"param":{"show_array":1,"gas_goes_into_solution":1,"calibr_li":2}}</v>
+      </c>
+      <c r="J6" t="s">
+        <v>58</v>
       </c>
     </row>
-    <row r="7" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -9018,8 +10680,11 @@
       <c r="I7" s="2">
         <v>50</v>
       </c>
+      <c r="J7" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="8" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
@@ -9038,8 +10703,11 @@
       <c r="I8" s="2">
         <v>200</v>
       </c>
+      <c r="J8" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="9" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
@@ -9059,8 +10727,20 @@
         <f>[1]!encode_linspace(1,I8,20)</f>
         <v>[1,10.95,20.9,30.85,40.8,50.75,60.7,70.65,80.6,90.55,100.5,110.45,120.4,130.35,140.3,150.25,160.2,170.15,180.1,190.05,200]</v>
       </c>
+      <c r="J9" t="s">
+        <v>58</v>
+      </c>
+      <c r="T9" t="s">
+        <v>59</v>
+      </c>
+      <c r="U9" t="s">
+        <v>60</v>
+      </c>
+      <c r="V9" t="s">
+        <v>61</v>
+      </c>
     </row>
-    <row r="10" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>7</v>
       </c>
@@ -9083,10 +10763,10 @@
       </c>
       <c r="J10" s="5">
         <f t="array" ref="J10:R10">[1]!well_ksep_full_d($I$3,$I$4,$I$10,$I$6,$I$7)</f>
-        <v>0.996</v>
+        <v>0.997</v>
       </c>
       <c r="K10" s="5">
-        <v>0.96399999999999997</v>
+        <v>0.97299999999999998</v>
       </c>
       <c r="L10" s="5">
         <v>0.88600000000000001</v>
@@ -9095,22 +10775,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":1,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N10" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":45.322,"pb_atma":58.596,"t_res_C":80,"bob_m3m3":1.091,"muob_cP":1.032,"PVT_corr_set":0,"q_liq_sm3day":2,"fw_perc":10,"rp_m3m3":45.322}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":45.279,"pb_atma":58.563,"t_res_C":80,"bob_m3m3":1.091,"muob_cP":1.031,"PVT_corr_set":0,"q_liq_sm3day":2,"fw_perc":10,"rp_m3m3":45.279}</v>
       </c>
       <c r="O10" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":66.1}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":66.156}</v>
       </c>
       <c r="P10" s="5">
-        <v>66.099999999999994</v>
+        <v>66.156000000000006</v>
       </c>
       <c r="Q10" s="5">
-        <v>0.23200000000000001</v>
+        <v>0.23300000000000001</v>
       </c>
       <c r="R10" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":47.041,"pb_atma":59.988,"t_res_C":80,"bob_m3m3":1.094,"muob_cP":1.027,"PVT_corr_set":0,"q_liq_sm3day":2,"fw_perc":10,"rp_m3m3":47.041}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":46.677,"pb_atma":59.605,"t_res_C":80,"bob_m3m3":1.093,"muob_cP":1.031,"PVT_corr_set":0,"q_liq_sm3day":2,"fw_perc":10,"rp_m3m3":46.677}</v>
+      </c>
+      <c r="S10" t="s">
+        <v>58</v>
+      </c>
+      <c r="T10" cm="1">
+        <f t="array" ref="T10">[1]!feed_gas_fraction_d($I$3,$I$4,I10)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U10" cm="1">
+        <f t="array" ref="U10">[1]!feed_gas_fraction_d($I$3,$I$4,N10)</f>
+        <v>9.7236563602478912E-3</v>
+      </c>
+      <c r="V10" cm="1">
+        <f t="array" ref="V10">[1]!feed_gas_fraction_d($I$3,$I$4,R10)</f>
+        <v>2.5533933853236015E-2</v>
       </c>
     </row>
-    <row r="11" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>8</v>
       </c>
@@ -9130,34 +10825,49 @@
       </c>
       <c r="J11" s="5">
         <f t="array" ref="J11:R11">[1]!well_ksep_full_d($I$3,$I$4,$I$11,$I$6,$I$7)</f>
-        <v>0.97199999999999998</v>
+        <v>0.97299999999999998</v>
       </c>
       <c r="K11" s="5">
-        <v>0.82899999999999996</v>
+        <v>0.83699999999999997</v>
       </c>
       <c r="L11" s="5">
-        <v>0.83299999999999996</v>
+        <v>0.83399999999999996</v>
       </c>
       <c r="M11" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":10.95,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N11" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":46.295,"pb_atma":59.485,"t_res_C":80,"bob_m3m3":1.093,"muob_cP":1.035,"PVT_corr_set":0,"q_liq_sm3day":21.9,"fw_perc":10,"rp_m3m3":46.295}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":46.236,"pb_atma":59.434,"t_res_C":80,"bob_m3m3":1.093,"muob_cP":1.034,"PVT_corr_set":0,"q_liq_sm3day":21.9,"fw_perc":10,"rp_m3m3":46.236}</v>
       </c>
       <c r="O11" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":707.334}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":708.286}</v>
       </c>
       <c r="P11" s="5">
-        <v>707.33399999999995</v>
+        <v>708.28599999999994</v>
       </c>
       <c r="Q11" s="5">
-        <v>2.2229999999999999</v>
+        <v>2.2410000000000001</v>
       </c>
       <c r="R11" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":52.069,"pb_atma":65.216,"t_res_C":80,"bob_m3m3":1.101,"muob_cP":0.977,"PVT_corr_set":0,"q_liq_sm3day":21.9,"fw_perc":10,"rp_m3m3":52.069}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":51.756,"pb_atma":64.898,"t_res_C":80,"bob_m3m3":1.1,"muob_cP":0.98,"PVT_corr_set":0,"q_liq_sm3day":21.9,"fw_perc":10,"rp_m3m3":51.756}</v>
+      </c>
+      <c r="S11" t="s">
+        <v>58</v>
+      </c>
+      <c r="T11" cm="1">
+        <f t="array" ref="T11">[1]!feed_gas_fraction_d($I$3,$I$4,I11)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U11" cm="1">
+        <f t="array" ref="U11">[1]!feed_gas_fraction_d($I$3,$I$4,N11)</f>
+        <v>2.2845064602382593E-2</v>
+      </c>
+      <c r="V11" cm="1">
+        <f t="array" ref="V11">[1]!feed_gas_fraction_d($I$3,$I$4,R11)</f>
+        <v>9.9050458581768572E-2</v>
       </c>
     </row>
-    <row r="12" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>9</v>
       </c>
@@ -9178,10 +10888,10 @@
       </c>
       <c r="J12" s="5">
         <f t="array" ref="J12:R12">[1]!well_ksep_full_d($I$3,$I$4,$I$12,$I$6,$I$7)</f>
-        <v>0.93899999999999995</v>
+        <v>0.94099999999999995</v>
       </c>
       <c r="K12" s="5">
-        <v>0.73099999999999998</v>
+        <v>0.73799999999999999</v>
       </c>
       <c r="L12" s="5">
         <v>0.77500000000000002</v>
@@ -9190,22 +10900,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":20.9,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N12" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":47.561,"pb_atma":60.743,"t_res_C":80,"bob_m3m3":1.094,"muob_cP":1.029,"PVT_corr_set":0,"q_liq_sm3day":41.8,"fw_perc":10,"rp_m3m3":47.561}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":47.489,"pb_atma":60.677,"t_res_C":80,"bob_m3m3":1.094,"muob_cP":1.029,"PVT_corr_set":0,"q_liq_sm3day":41.8,"fw_perc":10,"rp_m3m3":47.489}</v>
       </c>
       <c r="O12" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":1305.449}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":1307.805}</v>
       </c>
       <c r="P12" s="5">
-        <v>1305.4490000000001</v>
+        <v>1307.8050000000001</v>
       </c>
       <c r="Q12" s="5">
-        <v>3.37</v>
+        <v>3.4159999999999999</v>
       </c>
       <c r="R12" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":55.739,"pb_atma":68.949,"t_res_C":80,"bob_m3m3":1.106,"muob_cP":0.947,"PVT_corr_set":0,"q_liq_sm3day":41.8,"fw_perc":10,"rp_m3m3":55.739}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":55.464,"pb_atma":68.675,"t_res_C":80,"bob_m3m3":1.105,"muob_cP":0.949,"PVT_corr_set":0,"q_liq_sm3day":41.8,"fw_perc":10,"rp_m3m3":55.464}</v>
+      </c>
+      <c r="S12" t="s">
+        <v>58</v>
+      </c>
+      <c r="T12" cm="1">
+        <f t="array" ref="T12">[1]!feed_gas_fraction_d($I$3,$I$4,I12)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U12" cm="1">
+        <f t="array" ref="U12">[1]!feed_gas_fraction_d($I$3,$I$4,N12)</f>
+        <v>4.1094197807267863E-2</v>
+      </c>
+      <c r="V12" cm="1">
+        <f t="array" ref="V12">[1]!feed_gas_fraction_d($I$3,$I$4,R12)</f>
+        <v>0.14583284377950637</v>
       </c>
     </row>
-    <row r="13" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>10</v>
       </c>
@@ -9225,10 +10950,10 @@
       </c>
       <c r="J13" s="5">
         <f t="array" ref="J13:R13">[1]!well_ksep_full_d($I$3,$I$4,$I$13,$I$6,$I$7)</f>
-        <v>0.9</v>
+        <v>0.90200000000000002</v>
       </c>
       <c r="K13" s="5">
-        <v>0.65200000000000002</v>
+        <v>0.65900000000000003</v>
       </c>
       <c r="L13" s="5">
         <v>0.71299999999999997</v>
@@ -9237,22 +10962,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":30.85,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N13" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":49.112,"pb_atma":62.287,"t_res_C":80,"bob_m3m3":1.097,"muob_cP":1.02,"PVT_corr_set":0,"q_liq_sm3day":61.7,"fw_perc":10,"rp_m3m3":49.112}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":49.03,"pb_atma":62.208,"t_res_C":80,"bob_m3m3":1.097,"muob_cP":1.02,"PVT_corr_set":0,"q_liq_sm3day":61.7,"fw_perc":10,"rp_m3m3":49.03}</v>
       </c>
       <c r="O13" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":1845.406}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":1849.601}</v>
       </c>
       <c r="P13" s="5">
-        <v>1845.4059999999999</v>
+        <v>1849.6010000000001</v>
       </c>
       <c r="Q13" s="5">
-        <v>3.3809999999999998</v>
+        <v>3.4630000000000001</v>
       </c>
       <c r="R13" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":58.678,"pb_atma":71.858,"t_res_C":80,"bob_m3m3":1.11,"muob_cP":0.927,"PVT_corr_set":0,"q_liq_sm3day":61.7,"fw_perc":10,"rp_m3m3":58.678}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":58.432,"pb_atma":71.615,"t_res_C":80,"bob_m3m3":1.11,"muob_cP":0.929,"PVT_corr_set":0,"q_liq_sm3day":61.7,"fw_perc":10,"rp_m3m3":58.432}</v>
+      </c>
+      <c r="S13" t="s">
+        <v>58</v>
+      </c>
+      <c r="T13" cm="1">
+        <f t="array" ref="T13">[1]!feed_gas_fraction_d($I$3,$I$4,I13)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U13" cm="1">
+        <f t="array" ref="U13">[1]!feed_gas_fraction_d($I$3,$I$4,N13)</f>
+        <v>6.2777248767335814E-2</v>
+      </c>
+      <c r="V13" cm="1">
+        <f t="array" ref="V13">[1]!feed_gas_fraction_d($I$3,$I$4,R13)</f>
+        <v>0.1794397586713847</v>
       </c>
     </row>
-    <row r="14" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>11</v>
       </c>
@@ -9272,34 +11012,49 @@
       </c>
       <c r="J14" s="5">
         <f t="array" ref="J14:R14">[1]!well_ksep_full_d($I$3,$I$4,$I$14,$I$6,$I$7)</f>
-        <v>0.86199999999999999</v>
+        <v>0.86499999999999999</v>
       </c>
       <c r="K14" s="5">
-        <v>0.60699999999999998</v>
+        <v>0.61299999999999999</v>
       </c>
       <c r="L14" s="5">
-        <v>0.65</v>
+        <v>0.65100000000000002</v>
       </c>
       <c r="M14" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":40.8,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N14" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":50.564,"pb_atma":63.777,"t_res_C":80,"bob_m3m3":1.099,"muob_cP":1.008,"PVT_corr_set":0,"q_liq_sm3day":81.6,"fw_perc":10,"rp_m3m3":50.564}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":50.47,"pb_atma":63.685,"t_res_C":80,"bob_m3m3":1.099,"muob_cP":1.008,"PVT_corr_set":0,"q_liq_sm3day":81.6,"fw_perc":10,"rp_m3m3":50.47}</v>
       </c>
       <c r="O14" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":2336.113}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":2342.613}</v>
       </c>
       <c r="P14" s="5">
-        <v>2336.1129999999998</v>
+        <v>2342.6129999999998</v>
       </c>
       <c r="Q14" s="5">
-        <v>2.4300000000000002</v>
+        <v>2.5569999999999999</v>
       </c>
       <c r="R14" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":60.364,"pb_atma":73.527,"t_res_C":80,"bob_m3m3":1.112,"muob_cP":0.916,"PVT_corr_set":0,"q_liq_sm3day":81.6,"fw_perc":10,"rp_m3m3":60.364}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":60.135,"pb_atma":73.3,"t_res_C":80,"bob_m3m3":1.112,"muob_cP":0.918,"PVT_corr_set":0,"q_liq_sm3day":81.6,"fw_perc":10,"rp_m3m3":60.135}</v>
+      </c>
+      <c r="S14" t="s">
+        <v>58</v>
+      </c>
+      <c r="T14" cm="1">
+        <f t="array" ref="T14">[1]!feed_gas_fraction_d($I$3,$I$4,I14)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U14" cm="1">
+        <f t="array" ref="U14">[1]!feed_gas_fraction_d($I$3,$I$4,N14)</f>
+        <v>8.2885857814671157E-2</v>
+      </c>
+      <c r="V14" cm="1">
+        <f t="array" ref="V14">[1]!feed_gas_fraction_d($I$3,$I$4,R14)</f>
+        <v>0.19772138038641024</v>
       </c>
     </row>
-    <row r="15" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>12</v>
       </c>
@@ -9319,34 +11074,49 @@
       </c>
       <c r="J15" s="5">
         <f t="array" ref="J15:R15">[1]!well_ksep_full_d($I$3,$I$4,$I$15,$I$6,$I$7)</f>
-        <v>0.81399999999999995</v>
+        <v>0.81699999999999995</v>
       </c>
       <c r="K15" s="5">
-        <v>0.55400000000000005</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="L15" s="5">
-        <v>0.58399999999999996</v>
+        <v>0.58499999999999996</v>
       </c>
       <c r="M15" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":50.75,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N15" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":52.414,"pb_atma":65.655,"t_res_C":80,"bob_m3m3":1.101,"muob_cP":0.994,"PVT_corr_set":0,"q_liq_sm3day":101.5,"fw_perc":10,"rp_m3m3":52.414}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":52.31,"pb_atma":65.554,"t_res_C":80,"bob_m3m3":1.101,"muob_cP":0.994,"PVT_corr_set":0,"q_liq_sm3day":101.5,"fw_perc":10,"rp_m3m3":52.31}</v>
       </c>
       <c r="O15" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":2740.863}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":2749.76}</v>
       </c>
       <c r="P15" s="5">
-        <v>2740.8629999999998</v>
+        <v>2749.76</v>
       </c>
       <c r="Q15" s="5">
-        <v>-0.20200000000000001</v>
+        <v>-2.8000000000000001E-2</v>
       </c>
       <c r="R15" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":62.337,"pb_atma":75.45,"t_res_C":80,"bob_m3m3":1.115,"muob_cP":0.905,"PVT_corr_set":0,"q_liq_sm3day":101.5,"fw_perc":10,"rp_m3m3":62.337}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":62.128,"pb_atma":75.248,"t_res_C":80,"bob_m3m3":1.115,"muob_cP":0.906,"PVT_corr_set":0,"q_liq_sm3day":101.5,"fw_perc":10,"rp_m3m3":62.128}</v>
+      </c>
+      <c r="S15" t="s">
+        <v>58</v>
+      </c>
+      <c r="T15" cm="1">
+        <f t="array" ref="T15">[1]!feed_gas_fraction_d($I$3,$I$4,I15)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U15" cm="1">
+        <f t="array" ref="U15">[1]!feed_gas_fraction_d($I$3,$I$4,N15)</f>
+        <v>0.10732774085061607</v>
+      </c>
+      <c r="V15" cm="1">
+        <f t="array" ref="V15">[1]!feed_gas_fraction_d($I$3,$I$4,R15)</f>
+        <v>0.21797774972556341</v>
       </c>
     </row>
-    <row r="16" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>13</v>
       </c>
@@ -9357,7 +11127,7 @@
         <v>28</v>
       </c>
       <c r="F16" s="2">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="H16" s="5">
         <v>60.7</v>
@@ -9368,34 +11138,49 @@
       </c>
       <c r="J16" s="5">
         <f t="array" ref="J16:R16">[1]!well_ksep_full_d($I$3,$I$4,$I$16,$I$6,$I$7)</f>
-        <v>0.70299999999999996</v>
+        <v>0.73599999999999999</v>
       </c>
       <c r="K16" s="5">
-        <v>0.46400000000000002</v>
+        <v>0.51500000000000001</v>
       </c>
       <c r="L16" s="5">
-        <v>0.44700000000000001</v>
+        <v>0.45500000000000002</v>
       </c>
       <c r="M16" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":60.7,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N16" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":58.417,"pb_atma":71.924,"t_res_C":80,"bob_m3m3":1.11,"muob_cP":0.932,"PVT_corr_set":0,"q_liq_sm3day":121.4,"fw_perc":10,"rp_m3m3":58.417}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":57.173,"pb_atma":70.698,"t_res_C":80,"bob_m3m3":1.108,"muob_cP":0.939,"PVT_corr_set":0,"q_liq_sm3day":121.4,"fw_perc":10,"rp_m3m3":57.173}</v>
       </c>
       <c r="O16" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":2615.188}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":2747.19}</v>
       </c>
       <c r="P16" s="5">
-        <v>2615.1880000000001</v>
+        <v>2747.19</v>
       </c>
       <c r="Q16" s="5">
-        <v>-13.199</v>
+        <v>-10.619</v>
       </c>
       <c r="R16" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":69.043,"pb_atma":82.216,"t_res_C":80,"bob_m3m3":1.125,"muob_cP":0.85,"PVT_corr_set":0,"q_liq_sm3day":121.4,"fw_perc":10,"rp_m3m3":69.043}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":67.14,"pb_atma":80.379,"t_res_C":80,"bob_m3m3":1.122,"muob_cP":0.86,"PVT_corr_set":0,"q_liq_sm3day":121.4,"fw_perc":10,"rp_m3m3":67.14}</v>
+      </c>
+      <c r="S16" t="s">
+        <v>58</v>
+      </c>
+      <c r="T16" cm="1">
+        <f t="array" ref="T16">[1]!feed_gas_fraction_d($I$3,$I$4,I16)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U16" cm="1">
+        <f t="array" ref="U16">[1]!feed_gas_fraction_d($I$3,$I$4,N16)</f>
+        <v>0.16843619621973591</v>
+      </c>
+      <c r="V16" cm="1">
+        <f t="array" ref="V16">[1]!feed_gas_fraction_d($I$3,$I$4,R16)</f>
+        <v>0.26653454983912028</v>
       </c>
     </row>
-    <row r="17" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:22" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>14</v>
       </c>
@@ -9406,7 +11191,9 @@
       <c r="E17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F17" s="2"/>
+      <c r="F17" s="2">
+        <v>200</v>
+      </c>
       <c r="H17" s="5">
         <v>70.650000000000006</v>
       </c>
@@ -9416,34 +11203,49 @@
       </c>
       <c r="J17" s="5">
         <f t="array" ref="J17:R17">[1]!well_ksep_full_d($I$3,$I$4,$I$17,$I$6,$I$7)</f>
-        <v>0.52600000000000002</v>
+        <v>0.629</v>
       </c>
       <c r="K17" s="5">
-        <v>0.34899999999999998</v>
+        <v>0.47599999999999998</v>
       </c>
       <c r="L17" s="5">
-        <v>0.27200000000000002</v>
+        <v>0.29099999999999998</v>
       </c>
       <c r="M17" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":70.65,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N17" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":70.205,"pb_atma":83.993,"t_res_C":80,"bob_m3m3":1.126,"muob_cP":0.83,"PVT_corr_set":0,"q_liq_sm3day":141.3,"fw_perc":10,"rp_m3m3":70.205}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":66.169,"pb_atma":80.056,"t_res_C":80,"bob_m3m3":1.121,"muob_cP":0.852,"PVT_corr_set":0,"q_liq_sm3day":141.3,"fw_perc":10,"rp_m3m3":66.169}</v>
       </c>
       <c r="O17" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":1527.195}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":2032.719}</v>
       </c>
       <c r="P17" s="5">
-        <v>1527.1949999999999</v>
+        <v>2032.7190000000001</v>
       </c>
       <c r="Q17" s="5">
-        <v>-45.003</v>
+        <v>-35.122999999999998</v>
       </c>
       <c r="R17" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":79.558,"pb_atma":92.652,"t_res_C":80,"bob_m3m3":1.14,"muob_cP":0.776,"PVT_corr_set":0,"q_liq_sm3day":141.3,"fw_perc":10,"rp_m3m3":79.558}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":74.821,"pb_atma":88.148,"t_res_C":80,"bob_m3m3":1.133,"muob_cP":0.799,"PVT_corr_set":0,"q_liq_sm3day":141.3,"fw_perc":10,"rp_m3m3":74.821}</v>
+      </c>
+      <c r="S17" t="s">
+        <v>58</v>
+      </c>
+      <c r="T17" cm="1">
+        <f t="array" ref="T17">[1]!feed_gas_fraction_d($I$3,$I$4,I17)</f>
+        <v>0.55350477167797996</v>
+      </c>
+      <c r="U17" cm="1">
+        <f t="array" ref="U17">[1]!feed_gas_fraction_d($I$3,$I$4,N17)</f>
+        <v>0.26179777427701612</v>
+      </c>
+      <c r="V17" cm="1">
+        <f t="array" ref="V17">[1]!feed_gas_fraction_d($I$3,$I$4,R17)</f>
+        <v>0.33024790287712152</v>
       </c>
     </row>
-    <row r="18" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
       <c r="E18" s="1" t="s">
         <v>30</v>
       </c>
@@ -9457,40 +11259,55 @@
       </c>
       <c r="J18" s="5">
         <f t="array" ref="J18:R18">[1]!well_ksep_full_d($I$3,$I$4,$I$18,$I$6,$I$7)</f>
-        <v>0.35</v>
+        <v>0.53100000000000003</v>
       </c>
       <c r="K18" s="5">
-        <v>0.251</v>
+        <v>0.44400000000000001</v>
       </c>
       <c r="L18" s="5">
-        <v>0.13200000000000001</v>
+        <v>0.158</v>
       </c>
       <c r="M18" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":80.6,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N18" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":83.627,"pb_atma":97.377,"t_res_C":80,"bob_m3m3":1.146,"muob_cP":0.738,"PVT_corr_set":0,"q_liq_sm3day":161.2,"fw_perc":10,"rp_m3m3":83.627}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":76.421,"pb_atma":90.415,"t_res_C":80,"bob_m3m3":1.135,"muob_cP":0.775,"PVT_corr_set":0,"q_liq_sm3day":161.2,"fw_perc":10,"rp_m3m3":76.421}</v>
       </c>
       <c r="O18" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":815.03}</v>
       </c>
       <c r="P18" s="5">
-        <v>-225.703</v>
+        <v>815.03</v>
       </c>
       <c r="Q18" s="5">
-        <v>-131.68600000000001</v>
+        <v>-69.463999999999999</v>
       </c>
       <c r="R18" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":89.472,"pb_atma":102.277,"t_res_C":80,"bob_m3m3":1.154,"muob_cP":0.72,"PVT_corr_set":0,"q_liq_sm3day":161.2,"fw_perc":10,"rp_m3m3":89.472}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":82.286,"pb_atma":95.488,"t_res_C":80,"bob_m3m3":1.144,"muob_cP":0.752,"PVT_corr_set":0,"q_liq_sm3day":161.2,"fw_perc":10,"rp_m3m3":82.286}</v>
+      </c>
+      <c r="S18" t="s">
+        <v>58</v>
+      </c>
+      <c r="T18" cm="1">
+        <f t="array" ref="T18">[1]!feed_gas_fraction_d($I$3,$I$4,I18)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U18" cm="1">
+        <f t="array" ref="U18">[1]!feed_gas_fraction_d($I$3,$I$4,N18)</f>
+        <v>0.34511980621007499</v>
+      </c>
+      <c r="V18" cm="1">
+        <f t="array" ref="V18">[1]!feed_gas_fraction_d($I$3,$I$4,R18)</f>
+        <v>0.3819379134772044</v>
       </c>
     </row>
-    <row r="19" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
       <c r="E19" s="1" t="s">
         <v>31</v>
       </c>
       <c r="F19" s="3" t="str">
         <f>[1]!encode_ESP_separation(F3,F4, F5, F6,F7, F8, F9, F10, F11, F12, F13, F14, F15, F16, F17, F18)</f>
-        <v>{"calc_mode":"by_correlation","natsep_model":"0","d_intake_mm":"92","d_cas_mm":"125","d_tub_mm":"72","pkv_period_ratio":"0.5","gassep_type":"0","gassep_qnom_sm3day":"200","param":{"show_array":1,"gas_goes_into_solution":1,"calibr_li":2}}</v>
+        <v>{"calc_mode":"by_correlation","natsep_model":0,"d_intake_mm":92,"d_cas_mm":125,"d_tub_mm":72,"pkv_period_ratio":0.5,"gassep_type":-1,"gassep_qnom_sm3day":200,"param":{"show_array":1,"gas_goes_into_solution":1,"calibr_li":2}}</v>
       </c>
       <c r="H19" s="5">
         <v>90.55</v>
@@ -9501,34 +11318,49 @@
       </c>
       <c r="J19" s="5">
         <f t="array" ref="J19:R19">[1]!well_ksep_full_d($I$3,$I$4,$I$19,$I$6,$I$7)</f>
-        <v>0.193</v>
+        <v>0.45100000000000001</v>
       </c>
       <c r="K19" s="5">
-        <v>0.16600000000000001</v>
+        <v>0.41599999999999998</v>
       </c>
       <c r="L19" s="5">
-        <v>3.3000000000000002E-2</v>
+        <v>0.06</v>
       </c>
       <c r="M19" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":90.55,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N19" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":97.138,"pb_atma":110.561,"t_res_C":80,"bob_m3m3":1.165,"muob_cP":0.664,"PVT_corr_set":0,"q_liq_sm3day":181.1,"fw_perc":10,"rp_m3m3":97.138}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":86.919,"pb_atma":100.755,"t_res_C":80,"bob_m3m3":1.15,"muob_cP":0.712,"PVT_corr_set":0,"q_liq_sm3day":181.1,"fw_perc":10,"rp_m3m3":86.919}</v>
       </c>
       <c r="O19" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P19" s="5">
-        <v>-2479.1370000000002</v>
+        <v>-808.11300000000006</v>
       </c>
       <c r="Q19" s="5">
         <v>-167.85499999999999</v>
       </c>
       <c r="R19" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":98.905,"pb_atma":111.285,"t_res_C":80,"bob_m3m3":1.168,"muob_cP":0.674,"PVT_corr_set":0,"q_liq_sm3day":181.1,"fw_perc":10,"rp_m3m3":98.905}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":89.568,"pb_atma":102.474,"t_res_C":80,"bob_m3m3":1.154,"muob_cP":0.715,"PVT_corr_set":0,"q_liq_sm3day":181.1,"fw_perc":10,"rp_m3m3":89.568}</v>
+      </c>
+      <c r="S19" t="s">
+        <v>58</v>
+      </c>
+      <c r="T19" cm="1">
+        <f t="array" ref="T19">[1]!feed_gas_fraction_d($I$3,$I$4,I19)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U19" cm="1">
+        <f t="array" ref="U19">[1]!feed_gas_fraction_d($I$3,$I$4,N19)</f>
+        <v>0.41273119641773265</v>
+      </c>
+      <c r="V19" cm="1">
+        <f t="array" ref="V19">[1]!feed_gas_fraction_d($I$3,$I$4,R19)</f>
+        <v>0.42503786661386767</v>
       </c>
     </row>
-    <row r="20" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H20" s="5">
         <v>100.5</v>
       </c>
@@ -9538,10 +11370,10 @@
       </c>
       <c r="J20" s="5">
         <f t="array" ref="J20:R20">[1]!well_ksep_full_d($I$3,$I$4,$I$20,$I$6,$I$7)</f>
-        <v>3.9E-2</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="K20" s="5">
-        <v>3.9E-2</v>
+        <v>0.39200000000000002</v>
       </c>
       <c r="L20" s="5">
         <v>0</v>
@@ -9550,22 +11382,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":100.5,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N20" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.8,"pb_atma":127.439,"t_res_C":80,"bob_m3m3":1.191,"muob_cP":0.585,"PVT_corr_set":0,"q_liq_sm3day":201,"fw_perc":10,"rp_m3m3":114.8}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":101.609,"pb_atma":113.836,"t_res_C":80,"bob_m3m3":1.172,"muob_cP":0.662,"PVT_corr_set":0,"q_liq_sm3day":201,"fw_perc":10,"rp_m3m3":101.609}</v>
       </c>
       <c r="O20" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P20" s="5">
-        <v>-5979.63</v>
+        <v>-3480.7289999999998</v>
       </c>
       <c r="Q20" s="5">
         <v>-225.976</v>
       </c>
       <c r="R20" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.8,"pb_atma":126.285,"t_res_C":80,"bob_m3m3":1.192,"muob_cP":0.604,"PVT_corr_set":0,"q_liq_sm3day":201,"fw_perc":10,"rp_m3m3":114.8}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":101.609,"pb_atma":113.836,"t_res_C":80,"bob_m3m3":1.172,"muob_cP":0.662,"PVT_corr_set":0,"q_liq_sm3day":201,"fw_perc":10,"rp_m3m3":101.609}</v>
+      </c>
+      <c r="S20" t="s">
+        <v>58</v>
+      </c>
+      <c r="T20" cm="1">
+        <f t="array" ref="T20">[1]!feed_gas_fraction_d($I$3,$I$4,I20)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U20" cm="1">
+        <f t="array" ref="U20">[1]!feed_gas_fraction_d($I$3,$I$4,N20)</f>
+        <v>0.48442215735325556</v>
+      </c>
+      <c r="V20" cm="1">
+        <f t="array" ref="V20">[1]!feed_gas_fraction_d($I$3,$I$4,R20)</f>
+        <v>0.48442215735325556</v>
       </c>
     </row>
-    <row r="21" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H21" s="5">
         <v>110.45</v>
       </c>
@@ -9575,10 +11422,10 @@
       </c>
       <c r="J21" s="5">
         <f t="array" ref="J21:R21">[1]!well_ksep_full_d($I$3,$I$4,$I$21,$I$6,$I$7)</f>
-        <v>3.6999999999999998E-2</v>
+        <v>0.373</v>
       </c>
       <c r="K21" s="5">
-        <v>3.6999999999999998E-2</v>
+        <v>0.373</v>
       </c>
       <c r="L21" s="5">
         <v>0</v>
@@ -9587,22 +11434,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":110.45,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N21" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.874,"pb_atma":126.355,"t_res_C":80,"bob_m3m3":1.192,"muob_cP":0.603,"PVT_corr_set":0,"q_liq_sm3day":220.9,"fw_perc":10,"rp_m3m3":114.874}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":102.351,"pb_atma":114.537,"t_res_C":80,"bob_m3m3":1.173,"muob_cP":0.658,"PVT_corr_set":0,"q_liq_sm3day":220.9,"fw_perc":10,"rp_m3m3":102.351}</v>
       </c>
       <c r="O21" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P21" s="5">
-        <v>-6489.3670000000002</v>
+        <v>-3973.998</v>
       </c>
       <c r="Q21" s="5">
         <v>-248.34899999999999</v>
       </c>
       <c r="R21" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.874,"pb_atma":126.355,"t_res_C":80,"bob_m3m3":1.192,"muob_cP":0.603,"PVT_corr_set":0,"q_liq_sm3day":220.9,"fw_perc":10,"rp_m3m3":114.874}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":102.351,"pb_atma":114.537,"t_res_C":80,"bob_m3m3":1.173,"muob_cP":0.658,"PVT_corr_set":0,"q_liq_sm3day":220.9,"fw_perc":10,"rp_m3m3":102.351}</v>
+      </c>
+      <c r="S21" t="s">
+        <v>58</v>
+      </c>
+      <c r="T21" cm="1">
+        <f t="array" ref="T21">[1]!feed_gas_fraction_d($I$3,$I$4,I21)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U21" cm="1">
+        <f t="array" ref="U21">[1]!feed_gas_fraction_d($I$3,$I$4,N21)</f>
+        <v>0.48771028188520732</v>
+      </c>
+      <c r="V21" cm="1">
+        <f t="array" ref="V21">[1]!feed_gas_fraction_d($I$3,$I$4,R21)</f>
+        <v>0.48771028188520732</v>
       </c>
     </row>
-    <row r="22" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H22" s="5">
         <v>120.4</v>
       </c>
@@ -9612,10 +11474,10 @@
       </c>
       <c r="J22" s="5">
         <f t="array" ref="J22:R22">[1]!well_ksep_full_d($I$3,$I$4,$I$22,$I$6,$I$7)</f>
-        <v>3.5999999999999997E-2</v>
+        <v>0.35599999999999998</v>
       </c>
       <c r="K22" s="5">
-        <v>3.5999999999999997E-2</v>
+        <v>0.35599999999999998</v>
       </c>
       <c r="L22" s="5">
         <v>0</v>
@@ -9624,22 +11486,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":120.4,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N22" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.937,"pb_atma":127.569,"t_res_C":80,"bob_m3m3":1.191,"muob_cP":0.584,"PVT_corr_set":0,"q_liq_sm3day":240.8,"fw_perc":10,"rp_m3m3":114.937}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":102.979,"pb_atma":115.13,"t_res_C":80,"bob_m3m3":1.174,"muob_cP":0.656,"PVT_corr_set":0,"q_liq_sm3day":240.8,"fw_perc":10,"rp_m3m3":102.979}</v>
       </c>
       <c r="O22" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P22" s="5">
-        <v>-7193.7539999999999</v>
+        <v>-4469.0510000000004</v>
       </c>
       <c r="Q22" s="5">
         <v>-270.72199999999998</v>
       </c>
       <c r="R22" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.937,"pb_atma":126.414,"t_res_C":80,"bob_m3m3":1.192,"muob_cP":0.603,"PVT_corr_set":0,"q_liq_sm3day":240.8,"fw_perc":10,"rp_m3m3":114.937}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":102.979,"pb_atma":115.13,"t_res_C":80,"bob_m3m3":1.174,"muob_cP":0.656,"PVT_corr_set":0,"q_liq_sm3day":240.8,"fw_perc":10,"rp_m3m3":102.979}</v>
+      </c>
+      <c r="S22" t="s">
+        <v>58</v>
+      </c>
+      <c r="T22" cm="1">
+        <f t="array" ref="T22">[1]!feed_gas_fraction_d($I$3,$I$4,I22)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U22" cm="1">
+        <f t="array" ref="U22">[1]!feed_gas_fraction_d($I$3,$I$4,N22)</f>
+        <v>0.49044918942208804</v>
+      </c>
+      <c r="V22" cm="1">
+        <f t="array" ref="V22">[1]!feed_gas_fraction_d($I$3,$I$4,R22)</f>
+        <v>0.49044918942208804</v>
       </c>
     </row>
-    <row r="23" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H23" s="5">
         <v>130.35</v>
       </c>
@@ -9649,10 +11526,10 @@
       </c>
       <c r="J23" s="5">
         <f t="array" ref="J23:R23">[1]!well_ksep_full_d($I$3,$I$4,$I$23,$I$6,$I$7)</f>
-        <v>3.4000000000000002E-2</v>
+        <v>0.34200000000000003</v>
       </c>
       <c r="K23" s="5">
-        <v>3.4000000000000002E-2</v>
+        <v>0.34200000000000003</v>
       </c>
       <c r="L23" s="5">
         <v>0</v>
@@ -9661,22 +11538,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":130.35,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N23" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.99,"pb_atma":126.464,"t_res_C":80,"bob_m3m3":1.192,"muob_cP":0.603,"PVT_corr_set":0,"q_liq_sm3day":260.7,"fw_perc":10,"rp_m3m3":114.99}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":103.509,"pb_atma":115.63,"t_res_C":80,"bob_m3m3":1.175,"muob_cP":0.653,"PVT_corr_set":0,"q_liq_sm3day":260.7,"fw_perc":10,"rp_m3m3":103.509}</v>
       </c>
       <c r="O23" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P23" s="5">
-        <v>-7686.0879999999997</v>
+        <v>-4963.6130000000003</v>
       </c>
       <c r="Q23" s="5">
         <v>-293.09399999999999</v>
       </c>
       <c r="R23" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":114.99,"pb_atma":126.464,"t_res_C":80,"bob_m3m3":1.192,"muob_cP":0.603,"PVT_corr_set":0,"q_liq_sm3day":260.7,"fw_perc":10,"rp_m3m3":114.99}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":103.509,"pb_atma":115.63,"t_res_C":80,"bob_m3m3":1.175,"muob_cP":0.653,"PVT_corr_set":0,"q_liq_sm3day":260.7,"fw_perc":10,"rp_m3m3":103.509}</v>
+      </c>
+      <c r="S23" t="s">
+        <v>58</v>
+      </c>
+      <c r="T23" cm="1">
+        <f t="array" ref="T23">[1]!feed_gas_fraction_d($I$3,$I$4,I23)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U23" cm="1">
+        <f t="array" ref="U23">[1]!feed_gas_fraction_d($I$3,$I$4,N23)</f>
+        <v>0.49272556975681142</v>
+      </c>
+      <c r="V23" cm="1">
+        <f t="array" ref="V23">[1]!feed_gas_fraction_d($I$3,$I$4,R23)</f>
+        <v>0.49272556975681142</v>
       </c>
     </row>
-    <row r="24" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H24" s="5">
         <v>140.30000000000001</v>
       </c>
@@ -9686,10 +11578,10 @@
       </c>
       <c r="J24" s="5">
         <f t="array" ref="J24:R24">[1]!well_ksep_full_d($I$3,$I$4,$I$24,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.33</v>
       </c>
       <c r="K24" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.33</v>
       </c>
       <c r="L24" s="5">
         <v>0</v>
@@ -9698,22 +11590,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":140.3,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N24" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.503,"pb_atma":130.723,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":280.6,"fw_perc":10,"rp_m3m3":119.503}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":107.316,"pb_atma":120.307,"t_res_C":80,"bob_m3m3":1.18,"muob_cP":0.617,"PVT_corr_set":0,"q_liq_sm3day":280.6,"fw_perc":10,"rp_m3m3":107.316}</v>
       </c>
       <c r="O24" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P24" s="5">
-        <v>-9428.58</v>
+        <v>-6435.6469999999999</v>
       </c>
       <c r="Q24" s="5">
         <v>-332.255</v>
       </c>
       <c r="R24" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.503,"pb_atma":130.723,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":280.6,"fw_perc":10,"rp_m3m3":119.503}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":107.316,"pb_atma":119.222,"t_res_C":80,"bob_m3m3":1.181,"muob_cP":0.637,"PVT_corr_set":0,"q_liq_sm3day":280.6,"fw_perc":10,"rp_m3m3":107.316}</v>
+      </c>
+      <c r="S24" t="s">
+        <v>58</v>
+      </c>
+      <c r="T24" cm="1">
+        <f t="array" ref="T24">[1]!feed_gas_fraction_d($I$3,$I$4,I24)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U24" cm="1">
+        <f t="array" ref="U24">[1]!feed_gas_fraction_d($I$3,$I$4,N24)</f>
+        <v>0.51076729949079169</v>
+      </c>
+      <c r="V24" cm="1">
+        <f t="array" ref="V24">[1]!feed_gas_fraction_d($I$3,$I$4,R24)</f>
+        <v>0.50860666940773758</v>
       </c>
     </row>
-    <row r="25" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H25" s="5">
         <v>150.25</v>
       </c>
@@ -9723,10 +11630,10 @@
       </c>
       <c r="J25" s="5">
         <f t="array" ref="J25:R25">[1]!well_ksep_full_d($I$3,$I$4,$I$25,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.32</v>
       </c>
       <c r="K25" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.32</v>
       </c>
       <c r="L25" s="5">
         <v>0</v>
@@ -9735,22 +11642,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":150.25,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N25" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.507,"pb_atma":131.925,"t_res_C":80,"bob_m3m3":1.198,"muob_cP":0.564,"PVT_corr_set":0,"q_liq_sm3day":300.5,"fw_perc":10,"rp_m3m3":119.507}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":107.692,"pb_atma":119.577,"t_res_C":80,"bob_m3m3":1.181,"muob_cP":0.635,"PVT_corr_set":0,"q_liq_sm3day":300.5,"fw_perc":10,"rp_m3m3":107.692}</v>
       </c>
       <c r="O25" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P25" s="5">
-        <v>-10230.709999999999</v>
+        <v>-6862.799</v>
       </c>
       <c r="Q25" s="5">
         <v>-355.81799999999998</v>
       </c>
       <c r="R25" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.507,"pb_atma":130.727,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":300.5,"fw_perc":10,"rp_m3m3":119.507}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":107.692,"pb_atma":119.577,"t_res_C":80,"bob_m3m3":1.181,"muob_cP":0.635,"PVT_corr_set":0,"q_liq_sm3day":300.5,"fw_perc":10,"rp_m3m3":107.692}</v>
+      </c>
+      <c r="S25" t="s">
+        <v>58</v>
+      </c>
+      <c r="T25" cm="1">
+        <f t="array" ref="T25">[1]!feed_gas_fraction_d($I$3,$I$4,I25)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U25" cm="1">
+        <f t="array" ref="U25">[1]!feed_gas_fraction_d($I$3,$I$4,N25)</f>
+        <v>0.51016877555079976</v>
+      </c>
+      <c r="V25" cm="1">
+        <f t="array" ref="V25">[1]!feed_gas_fraction_d($I$3,$I$4,R25)</f>
+        <v>0.51016877555079976</v>
       </c>
     </row>
-    <row r="26" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H26" s="5">
         <v>160.19999999999999</v>
       </c>
@@ -9760,10 +11682,10 @@
       </c>
       <c r="J26" s="5">
         <f t="array" ref="J26:R26">[1]!well_ksep_full_d($I$3,$I$4,$I$26,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.311</v>
       </c>
       <c r="K26" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.311</v>
       </c>
       <c r="L26" s="5">
         <v>0</v>
@@ -9772,22 +11694,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":160.2,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N26" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.51,"pb_atma":130.73,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":320.4,"fw_perc":10,"rp_m3m3":119.51}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.009,"pb_atma":119.877,"t_res_C":80,"bob_m3m3":1.182,"muob_cP":0.634,"PVT_corr_set":0,"q_liq_sm3day":320.4,"fw_perc":10,"rp_m3m3":108.009}</v>
       </c>
       <c r="O26" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P26" s="5">
-        <v>-10767.948</v>
+        <v>-7409.66</v>
       </c>
       <c r="Q26" s="5">
         <v>-379.38099999999997</v>
       </c>
       <c r="R26" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.51,"pb_atma":130.73,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":320.4,"fw_perc":10,"rp_m3m3":119.51}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.009,"pb_atma":119.877,"t_res_C":80,"bob_m3m3":1.182,"muob_cP":0.634,"PVT_corr_set":0,"q_liq_sm3day":320.4,"fw_perc":10,"rp_m3m3":108.009}</v>
+      </c>
+      <c r="S26" t="s">
+        <v>58</v>
+      </c>
+      <c r="T26" cm="1">
+        <f t="array" ref="T26">[1]!feed_gas_fraction_d($I$3,$I$4,I26)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U26" cm="1">
+        <f t="array" ref="U26">[1]!feed_gas_fraction_d($I$3,$I$4,N26)</f>
+        <v>0.51140404733152833</v>
+      </c>
+      <c r="V26" cm="1">
+        <f t="array" ref="V26">[1]!feed_gas_fraction_d($I$3,$I$4,R26)</f>
+        <v>0.51140404733152833</v>
       </c>
     </row>
-    <row r="27" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H27" s="5">
         <v>170.15</v>
       </c>
@@ -9797,10 +11734,10 @@
       </c>
       <c r="J27" s="5">
         <f t="array" ref="J27:R27">[1]!well_ksep_full_d($I$3,$I$4,$I$27,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.30399999999999999</v>
       </c>
       <c r="K27" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.30399999999999999</v>
       </c>
       <c r="L27" s="5">
         <v>0</v>
@@ -9809,22 +11746,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":170.15,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N27" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.513,"pb_atma":130.732,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":340.3,"fw_perc":10,"rp_m3m3":119.513}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.278,"pb_atma":120.13,"t_res_C":80,"bob_m3m3":1.182,"muob_cP":0.632,"PVT_corr_set":0,"q_liq_sm3day":340.3,"fw_perc":10,"rp_m3m3":108.278}</v>
       </c>
       <c r="O27" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P27" s="5">
-        <v>-11437.579</v>
+        <v>-7953.0540000000001</v>
       </c>
       <c r="Q27" s="5">
         <v>-402.94499999999999</v>
       </c>
       <c r="R27" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.513,"pb_atma":130.732,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":340.3,"fw_perc":10,"rp_m3m3":119.513}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.278,"pb_atma":120.13,"t_res_C":80,"bob_m3m3":1.182,"muob_cP":0.632,"PVT_corr_set":0,"q_liq_sm3day":340.3,"fw_perc":10,"rp_m3m3":108.278}</v>
+      </c>
+      <c r="S27" t="s">
+        <v>58</v>
+      </c>
+      <c r="T27" cm="1">
+        <f t="array" ref="T27">[1]!feed_gas_fraction_d($I$3,$I$4,I27)</f>
+        <v>0.55350477167797996</v>
+      </c>
+      <c r="U27" cm="1">
+        <f t="array" ref="U27">[1]!feed_gas_fraction_d($I$3,$I$4,N27)</f>
+        <v>0.512508622496747</v>
+      </c>
+      <c r="V27" cm="1">
+        <f t="array" ref="V27">[1]!feed_gas_fraction_d($I$3,$I$4,R27)</f>
+        <v>0.512508622496747</v>
       </c>
     </row>
-    <row r="28" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H28" s="5">
         <v>180.1</v>
       </c>
@@ -9834,10 +11786,10 @@
       </c>
       <c r="J28" s="5">
         <f t="array" ref="J28:R28">[1]!well_ksep_full_d($I$3,$I$4,$I$28,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="K28" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.29799999999999999</v>
       </c>
       <c r="L28" s="5">
         <v>0</v>
@@ -9846,22 +11798,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":180.1,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N28" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.515,"pb_atma":131.933,"t_res_C":80,"bob_m3m3":1.198,"muob_cP":0.564,"PVT_corr_set":0,"q_liq_sm3day":360.2,"fw_perc":10,"rp_m3m3":119.515}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.508,"pb_atma":120.347,"t_res_C":80,"bob_m3m3":1.182,"muob_cP":0.631,"PVT_corr_set":0,"q_liq_sm3day":360.2,"fw_perc":10,"rp_m3m3":108.508}</v>
       </c>
       <c r="O28" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P28" s="5">
-        <v>-12265.919</v>
+        <v>-8493.4290000000001</v>
       </c>
       <c r="Q28" s="5">
         <v>-426.50799999999998</v>
       </c>
       <c r="R28" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.515,"pb_atma":130.734,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":360.2,"fw_perc":10,"rp_m3m3":119.515}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.508,"pb_atma":120.347,"t_res_C":80,"bob_m3m3":1.182,"muob_cP":0.631,"PVT_corr_set":0,"q_liq_sm3day":360.2,"fw_perc":10,"rp_m3m3":108.508}</v>
+      </c>
+      <c r="S28" t="s">
+        <v>58</v>
+      </c>
+      <c r="T28" cm="1">
+        <f t="array" ref="T28">[1]!feed_gas_fraction_d($I$3,$I$4,I28)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U28" cm="1">
+        <f t="array" ref="U28">[1]!feed_gas_fraction_d($I$3,$I$4,N28)</f>
+        <v>0.513450629685963</v>
+      </c>
+      <c r="V28" cm="1">
+        <f t="array" ref="V28">[1]!feed_gas_fraction_d($I$3,$I$4,R28)</f>
+        <v>0.513450629685963</v>
       </c>
     </row>
-    <row r="29" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H29" s="5">
         <v>190.05</v>
       </c>
@@ -9871,10 +11838,10 @@
       </c>
       <c r="J29" s="5">
         <f t="array" ref="J29:R29">[1]!well_ksep_full_d($I$3,$I$4,$I$29,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.29199999999999998</v>
       </c>
       <c r="K29" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.29199999999999998</v>
       </c>
       <c r="L29" s="5">
         <v>0</v>
@@ -9883,22 +11850,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":190.05,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N29" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.517,"pb_atma":131.934,"t_res_C":80,"bob_m3m3":1.198,"muob_cP":0.564,"PVT_corr_set":0,"q_liq_sm3day":380.1,"fw_perc":10,"rp_m3m3":119.517}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.708,"pb_atma":120.535,"t_res_C":80,"bob_m3m3":1.183,"muob_cP":0.631,"PVT_corr_set":0,"q_liq_sm3day":380.1,"fw_perc":10,"rp_m3m3":108.708}</v>
       </c>
       <c r="O29" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P29" s="5">
-        <v>-12944.267</v>
+        <v>-9031.607</v>
       </c>
       <c r="Q29" s="5">
         <v>-450.07100000000003</v>
       </c>
       <c r="R29" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.517,"pb_atma":130.736,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":380.1,"fw_perc":10,"rp_m3m3":119.517}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.708,"pb_atma":120.535,"t_res_C":80,"bob_m3m3":1.183,"muob_cP":0.631,"PVT_corr_set":0,"q_liq_sm3day":380.1,"fw_perc":10,"rp_m3m3":108.708}</v>
+      </c>
+      <c r="S29" t="s">
+        <v>58</v>
+      </c>
+      <c r="T29" cm="1">
+        <f t="array" ref="T29">[1]!feed_gas_fraction_d($I$3,$I$4,I29)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U29" cm="1">
+        <f t="array" ref="U29">[1]!feed_gas_fraction_d($I$3,$I$4,N29)</f>
+        <v>0.51419031206811949</v>
+      </c>
+      <c r="V29" cm="1">
+        <f t="array" ref="V29">[1]!feed_gas_fraction_d($I$3,$I$4,R29)</f>
+        <v>0.51419031206811949</v>
       </c>
     </row>
-    <row r="30" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H30" s="5">
         <v>200</v>
       </c>
@@ -9908,10 +11890,10 @@
       </c>
       <c r="J30" s="5">
         <f t="array" ref="J30:R31">[1]!well_ksep_full_d($I$3,$I$4,$I$30,$I$6,$I$7)</f>
-        <v>3.0000000000000001E-3</v>
+        <v>0.28799999999999998</v>
       </c>
       <c r="K30" s="5">
-        <v>3.0000000000000001E-3</v>
+        <v>0.28799999999999998</v>
       </c>
       <c r="L30" s="5">
         <v>0</v>
@@ -9920,22 +11902,37 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":200,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="N30" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.519,"pb_atma":131.936,"t_res_C":80,"bob_m3m3":1.198,"muob_cP":0.564,"PVT_corr_set":0,"q_liq_sm3day":400,"fw_perc":10,"rp_m3m3":119.519}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.884,"pb_atma":120.702,"t_res_C":80,"bob_m3m3":1.183,"muob_cP":0.63,"PVT_corr_set":0,"q_liq_sm3day":400,"fw_perc":10,"rp_m3m3":108.884}</v>
       </c>
       <c r="O30" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661}</v>
       </c>
       <c r="P30" s="5">
-        <v>-13622.606</v>
+        <v>-9568.7350000000006</v>
       </c>
       <c r="Q30" s="5">
         <v>-473.63499999999999</v>
       </c>
       <c r="R30" s="5" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":119.519,"pb_atma":130.738,"t_res_C":80,"bob_m3m3":1.199,"muob_cP":0.583,"PVT_corr_set":0,"q_liq_sm3day":400,"fw_perc":10,"rp_m3m3":119.519}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":108.884,"pb_atma":120.702,"t_res_C":80,"bob_m3m3":1.183,"muob_cP":0.63,"PVT_corr_set":0,"q_liq_sm3day":400,"fw_perc":10,"rp_m3m3":108.884}</v>
+      </c>
+      <c r="S30" t="s">
+        <v>58</v>
+      </c>
+      <c r="T30" cm="1">
+        <f t="array" ref="T30">[1]!feed_gas_fraction_d($I$3,$I$4,I30)</f>
+        <v>0.55350477167798007</v>
+      </c>
+      <c r="U30" cm="1">
+        <f t="array" ref="U30">[1]!feed_gas_fraction_d($I$3,$I$4,N30)</f>
+        <v>0.51490847339588086</v>
+      </c>
+      <c r="V30" cm="1">
+        <f t="array" ref="V30">[1]!feed_gas_fraction_d($I$3,$I$4,R30)</f>
+        <v>0.51490847339588086</v>
       </c>
     </row>
-    <row r="31" spans="2:18" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5" t="str">
@@ -9965,8 +11962,11 @@
       <c r="R31" s="5" t="str">
         <v>fluid_gs</v>
       </c>
+      <c r="S31" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="34" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="34" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E34" s="1" t="s">
         <v>16</v>
       </c>
@@ -9974,7 +11974,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="35" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="35" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E35" s="1" t="s">
         <v>17</v>
       </c>
@@ -9982,7 +11982,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="36" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="36" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E36" s="1" t="s">
         <v>14</v>
       </c>
@@ -9991,16 +11991,16 @@
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":30,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
     </row>
-    <row r="37" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="37" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E37" s="1" t="s">
         <v>32</v>
       </c>
       <c r="F37" s="2" t="str">
         <f>gas_separation_json</f>
-        <v>{"calc_mode":"by_correlation","natsep_model":"0","d_intake_mm":"92","d_cas_mm":"125","d_tub_mm":"72","pkv_period_ratio":"0.5","gassep_type":"0","gassep_qnom_sm3day":"200","param":{"show_array":1,"gas_goes_into_solution":1,"calibr_li":2}}</v>
+        <v>{"calc_mode":"by_correlation","natsep_model":0,"d_intake_mm":92,"d_cas_mm":125,"d_tub_mm":72,"pkv_period_ratio":0.5,"gassep_type":-1,"gassep_qnom_sm3day":200,"param":{"show_array":1,"gas_goes_into_solution":1,"calibr_li":2}}</v>
       </c>
     </row>
-    <row r="38" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="38" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E38" s="1" t="s">
         <v>33</v>
       </c>
@@ -10008,7 +12008,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="39" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E39" s="1" t="s">
         <v>56</v>
       </c>
@@ -10016,40 +12016,40 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="40" spans="5:14" x14ac:dyDescent="0.25">
       <c r="E40" t="s">
         <v>57</v>
       </c>
       <c r="F40" s="3">
         <f t="array" ref="F40:N41">[1]!well_ksep_full_d(F34,F35,F36,F37,F38,F39)</f>
-        <v>0.90400000000000003</v>
+        <v>0.90600000000000003</v>
       </c>
       <c r="G40" s="3">
-        <v>0.65800000000000003</v>
+        <v>0.66500000000000004</v>
       </c>
       <c r="H40" s="3">
-        <v>0.71799999999999997</v>
+        <v>0.71899999999999997</v>
       </c>
       <c r="I40" s="3" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":30,"fw_perc":10,"rp_m3m3":120}</v>
       </c>
       <c r="J40" s="3" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":48.972,"pb_atma":62.145,"t_res_C":80,"bob_m3m3":1.096,"muob_cP":1.021,"PVT_corr_set":0,"q_liq_sm3day":60,"fw_perc":10,"rp_m3m3":48.972}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":48.89,"pb_atma":62.067,"t_res_C":80,"bob_m3m3":1.096,"muob_cP":1.021,"PVT_corr_set":0,"q_liq_sm3day":60,"fw_perc":10,"rp_m3m3":48.89}</v>
       </c>
       <c r="K40" s="3" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":120,"pb_atma":130,"t_res_C":80,"bob_m3m3":1.2,"muob_cP":0.6,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":10,"rp_m3m3":120,"q_gas_free_sm3day":1801.876}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":6.526,"pb_atma":11.571,"t_res_C":80,"bob_m3m3":1.04,"muob_cP":2.111,"PVT_corr_set":0,"q_liq_sm3day":0,"fw_perc":0,"rp_m3m3":7.661,"q_gas_free_sm3day":1805.899}</v>
       </c>
       <c r="L40" s="3">
-        <v>1801.876</v>
+        <v>1805.8989999999999</v>
       </c>
       <c r="M40" s="3">
-        <v>3.431</v>
+        <v>3.51</v>
       </c>
       <c r="N40" s="3" t="str">
-        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":58.45,"pb_atma":71.632,"t_res_C":80,"bob_m3m3":1.11,"muob_cP":0.929,"PVT_corr_set":0,"q_liq_sm3day":60,"fw_perc":10,"rp_m3m3":58.45}</v>
+        <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1.1,"rsb_m3m3":58.201,"pb_atma":71.386,"t_res_C":80,"bob_m3m3":1.109,"muob_cP":0.93,"PVT_corr_set":0,"q_liq_sm3day":60,"fw_perc":10,"rp_m3m3":58.201}</v>
       </c>
     </row>
-    <row r="41" spans="5:14" x14ac:dyDescent="0.4">
+    <row r="41" spans="5:14" x14ac:dyDescent="0.25">
       <c r="F41" s="3" t="str">
         <v>ksep_total_fr</v>
       </c>
@@ -10089,9 +12089,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA8F6952-8512-4B85-BDB2-56CC06FF34D9}">
   <sheetPr codeName="Лист2"/>
   <dimension ref="B4:E36"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>28</v>
       </c>
@@ -10099,7 +12099,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>36</v>
       </c>
@@ -10107,7 +12107,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>10</v>
       </c>
@@ -10115,7 +12115,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>37</v>
       </c>
@@ -10123,7 +12123,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>38</v>
       </c>
@@ -10132,7 +12132,7 @@
         <v>GDNK5</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>39</v>
       </c>
@@ -10140,7 +12140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>40</v>
       </c>
@@ -10148,7 +12148,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="11" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>41</v>
       </c>
@@ -10156,7 +12156,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>42</v>
       </c>
@@ -10164,7 +12164,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>35</v>
       </c>
@@ -10173,7 +12173,7 @@
         <v>[1,25.95,50.9,75.85,100.8,125.75,150.7,175.65,200.6,225.55,250.5,275.45,300.4,325.35,350.3,375.25,400.2,425.15,450.1,475.05,500]</v>
       </c>
     </row>
-    <row r="14" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>43</v>
       </c>
@@ -10182,7 +12182,7 @@
         <v>[0,0.05,0.1,0.15,0.2,0.25,0.3,0.35,0.4,0.45,0.5,0.55,0.6,0.65,0.7,0.75,0.8,0.85,0.9,0.95,1]</v>
       </c>
     </row>
-    <row r="15" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>44</v>
       </c>
@@ -10196,7 +12196,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16">
         <f t="array" ref="B16:B36">[1]!decode_json(C13)</f>
         <v>1</v>
@@ -10214,7 +12214,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17">
         <v>25.95</v>
       </c>
@@ -10230,7 +12230,7 @@
         <v>0.6298457675247221</v>
       </c>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18">
         <v>50.9</v>
       </c>
@@ -10246,13 +12246,13 @@
         <v>0.68898442009600003</v>
       </c>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19">
         <v>75.849999999999994</v>
       </c>
       <c r="C19">
         <f>[1]!ESP_gassep_ksep_d($C$4,$C$5,$B$19,$C$7)</f>
-        <v>0.85841925945936737</v>
+        <v>0.85841925945936748</v>
       </c>
       <c r="D19">
         <v>0.15</v>
@@ -10262,7 +12262,7 @@
         <v>0.73791840316599999</v>
       </c>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>100.8</v>
       </c>
@@ -10278,7 +12278,7 @@
         <v>0.78649188018600003</v>
       </c>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>125.75</v>
       </c>
@@ -10294,13 +12294,13 @@
         <v>0.82869092890600005</v>
       </c>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>150.69999999999999</v>
       </c>
       <c r="C22">
         <f>[1]!ESP_gassep_ksep_d($C$4,$C$5,$B$22,$C$7)</f>
-        <v>0.77637348447386989</v>
+        <v>0.77637348447387</v>
       </c>
       <c r="D22">
         <v>0.3</v>
@@ -10310,13 +12310,13 @@
         <v>0.85982152207599993</v>
       </c>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>175.65</v>
       </c>
       <c r="C23">
         <f>[1]!ESP_gassep_ksep_d($C$4,$C$5,$B$23,$C$7)</f>
-        <v>0.73940798366006733</v>
+        <v>0.73940798366006744</v>
       </c>
       <c r="D23">
         <v>0.35</v>
@@ -10326,7 +12326,7 @@
         <v>0.87650952744600008</v>
       </c>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>200.6</v>
       </c>
@@ -10342,7 +12342,7 @@
         <v>0.87670070776599995</v>
       </c>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>225.55</v>
       </c>
@@ -10358,7 +12358,7 @@
         <v>0.85966072078600009</v>
       </c>
     </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>250.5</v>
       </c>
@@ -10371,10 +12371,10 @@
       </c>
       <c r="E26">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$26,$C$6,$C$7)</f>
-        <v>0.8259751192560002</v>
+        <v>0.82597511925599998</v>
       </c>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>275.45</v>
       </c>
@@ -10387,10 +12387,10 @@
       </c>
       <c r="E27">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$27,$C$6,$C$7)</f>
-        <v>0.7775493509260003</v>
+        <v>0.77754935092600019</v>
       </c>
     </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>300.39999999999998</v>
       </c>
@@ -10403,10 +12403,10 @@
       </c>
       <c r="E28">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$28,$C$6,$C$7)</f>
-        <v>0.71760875854599993</v>
+        <v>0.71760875854600004</v>
       </c>
     </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>325.35000000000002</v>
       </c>
@@ -10419,10 +12419,10 @@
       </c>
       <c r="E29">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$29,$C$6,$C$7)</f>
-        <v>0.65069857986600033</v>
+        <v>0.6506985798660001</v>
       </c>
     </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30">
         <v>350.3</v>
       </c>
@@ -10435,10 +12435,10 @@
       </c>
       <c r="E30">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$30,$C$6,$C$7)</f>
-        <v>0.58268394763599962</v>
+        <v>0.58268394763600018</v>
       </c>
     </row>
-    <row r="31" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>375.25</v>
       </c>
@@ -10451,10 +12451,10 @@
       </c>
       <c r="E31">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$31,$C$6,$C$7)</f>
-        <v>0.52074988960600077</v>
+        <v>0.52074988960600022</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B32">
         <v>400.2</v>
       </c>
@@ -10467,10 +12467,10 @@
       </c>
       <c r="E32">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$32,$C$6,$C$7)</f>
-        <v>0.47340132852599986</v>
+        <v>0.47340132852600031</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33">
         <v>425.15</v>
       </c>
@@ -10483,10 +12483,10 @@
       </c>
       <c r="E33">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$33,$C$6,$C$7)</f>
-        <v>0.42574987164024719</v>
+        <v>0.42574987164025058</v>
       </c>
     </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34">
         <v>450.1</v>
       </c>
@@ -10499,10 +12499,10 @@
       </c>
       <c r="E34">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$34,$C$6,$C$7)</f>
-        <v>0.33170162999063563</v>
+        <v>0.3317016299906379</v>
       </c>
     </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35">
         <v>475.05</v>
       </c>
@@ -10515,10 +12515,10 @@
       </c>
       <c r="E35">
         <f>[1]!ESP_gassep_ksep_d($C$4,$D$35,$C$6,$C$7)</f>
-        <v>0.18978500611055324</v>
+        <v>0.18978500611055438</v>
       </c>
     </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>500</v>
       </c>
@@ -10543,10 +12543,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DAC09C0-00FB-4036-B6F8-3AB764A7C516}">
   <sheetPr codeName="Лист3"/>
-  <dimension ref="B3:D37"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <dimension ref="B3:E37"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>34</v>
       </c>
@@ -10554,7 +12554,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>47</v>
       </c>
@@ -10563,7 +12563,7 @@
         <v>[1,10.95,20.9,30.85,40.8,50.75,60.7,70.65,80.6,90.55,100.5,110.45,120.4,130.35,140.3,150.25,160.2,170.15,180.1,190.05,200]</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
@@ -10572,7 +12572,7 @@
         <v>[{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":1},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":10.95},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":20.9},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":30.85},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":40.8},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":50.75},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":60.7},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":70.65},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":80.6},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":90.55},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":100.5},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":110.45},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":120.4},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":130.35},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":140.3},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":150.25},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":160.2},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":170.15},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":180.1},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":190.05},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":100,"q_liq_sm3day":200}]</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>48</v>
       </c>
@@ -10580,7 +12580,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>49</v>
       </c>
@@ -10588,7 +12588,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>50</v>
       </c>
@@ -10596,7 +12596,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>51</v>
       </c>
@@ -10604,7 +12604,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>52</v>
       </c>
@@ -10612,7 +12612,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>22</v>
       </c>
@@ -10620,7 +12620,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>26</v>
       </c>
@@ -10628,7 +12628,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>27</v>
       </c>
@@ -10636,7 +12636,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>30</v>
       </c>
@@ -10644,7 +12644,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>54</v>
       </c>
@@ -10653,7 +12653,7 @@
         <v>{"p_atma":[50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50],"t_C":[50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50,50],"feed":[{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":22.764,"pb_atma":61.362,"t_res_C":90,"bob_m3m3":1.115,"muob_cP":1.251,"PVT_corr_set":0,"q_liq_sm3day":1,"fw_perc":0,"rp_m3m3":22.764},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":28.957,"pb_atma":75.037,"t_res_C":90,"bob_m3m3":1.129,"muob_cP":1.131,"PVT_corr_set":0,"q_liq_sm3day":10.95,"fw_perc":0,"rp_m3m3":28.957},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":33.91,"pb_atma":85.534,"t_res_C":90,"bob_m3m3":1.14,"muob_cP":1.056,"PVT_corr_set":0,"q_liq_sm3day":20.9,"fw_perc":0,"rp_m3m3":33.91},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":38.184,"pb_atma":94.422,"t_res_C":90,"bob_m3m3":1.15,"muob_cP":0.999,"PVT_corr_set":0,"q_liq_sm3day":30.85,"fw_perc":0,"rp_m3m3":38.184},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":41.957,"pb_atma":102.099,"t_res_C":90,"bob_m3m3":1.159,"muob_cP":0.956,"PVT_corr_set":0,"q_liq_sm3day":40.8,"fw_perc":0,"rp_m3m3":41.957},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":45.327,"pb_atma":108.932,"t_res_C":90,"bob_m3m3":1.167,"muob_cP":0.919,"PVT_corr_set":0,"q_liq_sm3day":50.75,"fw_perc":0,"rp_m3m3":45.327},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":48.359,"pb_atma":114.898,"t_res_C":90,"bob_m3m3":1.174,"muob_cP":0.892,"PVT_corr_set":0,"q_liq_sm3day":60.7,"fw_perc":0,"rp_m3m3":48.359},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":49.608,"pb_atma":117.354,"t_res_C":90,"bob_m3m3":1.177,"muob_cP":0.88,"PVT_corr_set":0,"q_liq_sm3day":70.65,"fw_perc":0,"rp_m3m3":49.608},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":52.037,"pb_atma":122.133,"t_res_C":90,"bob_m3m3":1.183,"muob_cP":0.859,"PVT_corr_set":0,"q_liq_sm3day":80.6,"fw_perc":0,"rp_m3m3":52.037},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":54.261,"pb_atma":126.495,"t_res_C":90,"bob_m3m3":1.188,"muob_cP":0.839,"PVT_corr_set":0,"q_liq_sm3day":90.55,"fw_perc":0,"rp_m3m3":54.261},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":56.299,"pb_atma":130.39,"t_res_C":90,"bob_m3m3":1.193,"muob_cP":0.825,"PVT_corr_set":0,"q_liq_sm3day":100.5,"fw_perc":0,"rp_m3m3":56.299},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":58.171,"pb_atma":133.967,"t_res_C":90,"bob_m3m3":1.198,"muob_cP":0.811,"PVT_corr_set":0,"q_liq_sm3day":110.45,"fw_perc":0,"rp_m3m3":58.171},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":59.89,"pb_atma":137.253,"t_res_C":90,"bob_m3m3":1.202,"muob_cP":0.799,"PVT_corr_set":0,"q_liq_sm3day":120.4,"fw_perc":0,"rp_m3m3":59.89},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":61.471,"pb_atma":140.273,"t_res_C":90,"bob_m3m3":1.206,"muob_cP":0.788,"PVT_corr_set":0,"q_liq_sm3day":130.35,"fw_perc":0,"rp_m3m3":61.471},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":62.925,"pb_atma":143.052,"t_res_C":90,"bob_m3m3":1.209,"muob_cP":0.777,"PVT_corr_set":0,"q_liq_sm3day":140.3,"fw_perc":0,"rp_m3m3":62.925},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":64.262,"pb_atma":145.565,"t_res_C":90,"bob_m3m3":1.212,"muob_cP":0.769,"PVT_corr_set":0,"q_liq_sm3day":150.25,"fw_perc":0,"rp_m3m3":64.262},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":65.492,"pb_atma":147.857,"t_res_C":90,"bob_m3m3":1.215,"muob_cP":0.762,"PVT_corr_set":0,"q_liq_sm3day":160.2,"fw_perc":0,"rp_m3m3":65.492},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":66.623,"pb_atma":149.964,"t_res_C":90,"bob_m3m3":1.218,"muob_cP":0.755,"PVT_corr_set":0,"q_liq_sm3day":170.15,"fw_perc":0,"rp_m3m3":66.623},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":67.662,"pb_atma":151.901,"t_res_C":90,"bob_m3m3":1.221,"muob_cP":0.749,"PVT_corr_set":0,"q_liq_sm3day":180.1,"fw_perc":0,"rp_m3m3":67.662},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":68.618,"pb_atma":153.681,"t_res_C":90,"bob_m3m3":1.223,"muob_cP":0.743,"PVT_corr_set":0,"q_liq_sm3day":190.05,"fw_perc":0,"rp_m3m3":68.618},{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":69.495,"pb_atma":155.315,"t_res_C":90,"bob_m3m3":1.225,"muob_cP":0.738,"PVT_corr_set":0,"q_liq_sm3day":200,"fw_perc":0,"rp_m3m3":69.495}],"k_sep":[0.98147,0.90277,0.83983,0.78552,0.73758,0.69476,0.65622,0.64035,0.60948,0.58123,0.55532,0.53154,0.50969,0.4896,0.47113,0.45414,0.43851,0.42414,0.41093,0.39879,0.38764]}</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.4">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>44</v>
       </c>
@@ -10661,7 +12661,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="17" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B17" s="5">
         <f t="array" ref="B17:B37">[1]!decode_json(C4)</f>
         <v>1</v>
@@ -10674,8 +12674,11 @@
         <f t="array" ref="D17:D37">[1]!decode_json([1]!decode_json(C15,,"feed",1))</f>
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":22.764,"pb_atma":61.362,"t_res_C":90,"bob_m3m3":1.115,"muob_cP":1.251,"PVT_corr_set":0,"q_liq_sm3day":1,"fw_perc":0,"rp_m3m3":22.764}</v>
       </c>
+      <c r="E17" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="18" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B18" s="5">
         <v>10.95</v>
       </c>
@@ -10685,8 +12688,11 @@
       <c r="D18" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":28.957,"pb_atma":75.037,"t_res_C":90,"bob_m3m3":1.129,"muob_cP":1.131,"PVT_corr_set":0,"q_liq_sm3day":10.95,"fw_perc":0,"rp_m3m3":28.957}</v>
       </c>
+      <c r="E18" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="19" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B19" s="5">
         <v>20.9</v>
       </c>
@@ -10696,8 +12702,11 @@
       <c r="D19" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":33.91,"pb_atma":85.534,"t_res_C":90,"bob_m3m3":1.14,"muob_cP":1.056,"PVT_corr_set":0,"q_liq_sm3day":20.9,"fw_perc":0,"rp_m3m3":33.91}</v>
       </c>
+      <c r="E19" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="20" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B20" s="5">
         <v>30.85</v>
       </c>
@@ -10707,8 +12716,11 @@
       <c r="D20" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":38.184,"pb_atma":94.422,"t_res_C":90,"bob_m3m3":1.15,"muob_cP":0.999,"PVT_corr_set":0,"q_liq_sm3day":30.85,"fw_perc":0,"rp_m3m3":38.184}</v>
       </c>
+      <c r="E20" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="21" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B21" s="5">
         <v>40.799999999999997</v>
       </c>
@@ -10718,8 +12730,11 @@
       <c r="D21" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":41.957,"pb_atma":102.099,"t_res_C":90,"bob_m3m3":1.159,"muob_cP":0.956,"PVT_corr_set":0,"q_liq_sm3day":40.8,"fw_perc":0,"rp_m3m3":41.957}</v>
       </c>
+      <c r="E21" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="22" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B22" s="5">
         <v>50.75</v>
       </c>
@@ -10729,8 +12744,11 @@
       <c r="D22" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":45.327,"pb_atma":108.932,"t_res_C":90,"bob_m3m3":1.167,"muob_cP":0.919,"PVT_corr_set":0,"q_liq_sm3day":50.75,"fw_perc":0,"rp_m3m3":45.327}</v>
       </c>
+      <c r="E22" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="23" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B23" s="5">
         <v>60.7</v>
       </c>
@@ -10740,8 +12758,11 @@
       <c r="D23" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":48.359,"pb_atma":114.898,"t_res_C":90,"bob_m3m3":1.174,"muob_cP":0.892,"PVT_corr_set":0,"q_liq_sm3day":60.7,"fw_perc":0,"rp_m3m3":48.359}</v>
       </c>
+      <c r="E23" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="24" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B24" s="5">
         <v>70.650000000000006</v>
       </c>
@@ -10751,8 +12772,11 @@
       <c r="D24" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":49.608,"pb_atma":117.354,"t_res_C":90,"bob_m3m3":1.177,"muob_cP":0.88,"PVT_corr_set":0,"q_liq_sm3day":70.65,"fw_perc":0,"rp_m3m3":49.608}</v>
       </c>
+      <c r="E24" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="25" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B25" s="5">
         <v>80.599999999999994</v>
       </c>
@@ -10762,8 +12786,11 @@
       <c r="D25" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":52.037,"pb_atma":122.133,"t_res_C":90,"bob_m3m3":1.183,"muob_cP":0.859,"PVT_corr_set":0,"q_liq_sm3day":80.6,"fw_perc":0,"rp_m3m3":52.037}</v>
       </c>
+      <c r="E25" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="26" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B26" s="5">
         <v>90.55</v>
       </c>
@@ -10773,8 +12800,11 @@
       <c r="D26" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":54.261,"pb_atma":126.495,"t_res_C":90,"bob_m3m3":1.188,"muob_cP":0.839,"PVT_corr_set":0,"q_liq_sm3day":90.55,"fw_perc":0,"rp_m3m3":54.261}</v>
       </c>
+      <c r="E26" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="27" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B27" s="5">
         <v>100.5</v>
       </c>
@@ -10784,8 +12814,11 @@
       <c r="D27" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":56.299,"pb_atma":130.39,"t_res_C":90,"bob_m3m3":1.193,"muob_cP":0.825,"PVT_corr_set":0,"q_liq_sm3day":100.5,"fw_perc":0,"rp_m3m3":56.299}</v>
       </c>
+      <c r="E27" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="28" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B28" s="5">
         <v>110.45</v>
       </c>
@@ -10795,8 +12828,11 @@
       <c r="D28" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":58.171,"pb_atma":133.967,"t_res_C":90,"bob_m3m3":1.198,"muob_cP":0.811,"PVT_corr_set":0,"q_liq_sm3day":110.45,"fw_perc":0,"rp_m3m3":58.171}</v>
       </c>
+      <c r="E28" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="29" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B29" s="5">
         <v>120.4</v>
       </c>
@@ -10806,8 +12842,11 @@
       <c r="D29" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":59.89,"pb_atma":137.253,"t_res_C":90,"bob_m3m3":1.202,"muob_cP":0.799,"PVT_corr_set":0,"q_liq_sm3day":120.4,"fw_perc":0,"rp_m3m3":59.89}</v>
       </c>
+      <c r="E29" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="30" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B30" s="5">
         <v>130.35</v>
       </c>
@@ -10817,8 +12856,11 @@
       <c r="D30" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":61.471,"pb_atma":140.273,"t_res_C":90,"bob_m3m3":1.206,"muob_cP":0.788,"PVT_corr_set":0,"q_liq_sm3day":130.35,"fw_perc":0,"rp_m3m3":61.471}</v>
       </c>
+      <c r="E30" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="31" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="31" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B31" s="5">
         <v>140.30000000000001</v>
       </c>
@@ -10828,8 +12870,11 @@
       <c r="D31" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":62.925,"pb_atma":143.052,"t_res_C":90,"bob_m3m3":1.209,"muob_cP":0.777,"PVT_corr_set":0,"q_liq_sm3day":140.3,"fw_perc":0,"rp_m3m3":62.925}</v>
       </c>
+      <c r="E31" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="32" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B32" s="5">
         <v>150.25</v>
       </c>
@@ -10839,8 +12884,11 @@
       <c r="D32" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":64.262,"pb_atma":145.565,"t_res_C":90,"bob_m3m3":1.212,"muob_cP":0.769,"PVT_corr_set":0,"q_liq_sm3day":150.25,"fw_perc":0,"rp_m3m3":64.262}</v>
       </c>
+      <c r="E32" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="33" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B33" s="5">
         <v>160.19999999999999</v>
       </c>
@@ -10850,8 +12898,11 @@
       <c r="D33" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":65.492,"pb_atma":147.857,"t_res_C":90,"bob_m3m3":1.215,"muob_cP":0.762,"PVT_corr_set":0,"q_liq_sm3day":160.2,"fw_perc":0,"rp_m3m3":65.492}</v>
       </c>
+      <c r="E33" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="34" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B34" s="5">
         <v>170.15</v>
       </c>
@@ -10861,8 +12912,11 @@
       <c r="D34" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":66.623,"pb_atma":149.964,"t_res_C":90,"bob_m3m3":1.218,"muob_cP":0.755,"PVT_corr_set":0,"q_liq_sm3day":170.15,"fw_perc":0,"rp_m3m3":66.623}</v>
       </c>
+      <c r="E34" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="35" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B35" s="5">
         <v>180.1</v>
       </c>
@@ -10872,8 +12926,11 @@
       <c r="D35" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":67.662,"pb_atma":151.901,"t_res_C":90,"bob_m3m3":1.221,"muob_cP":0.749,"PVT_corr_set":0,"q_liq_sm3day":180.1,"fw_perc":0,"rp_m3m3":67.662}</v>
       </c>
+      <c r="E35" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="36" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B36" s="5">
         <v>190.05</v>
       </c>
@@ -10883,8 +12940,11 @@
       <c r="D36" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":68.618,"pb_atma":153.681,"t_res_C":90,"bob_m3m3":1.223,"muob_cP":0.743,"PVT_corr_set":0,"q_liq_sm3day":190.05,"fw_perc":0,"rp_m3m3":68.618}</v>
       </c>
+      <c r="E36" t="s">
+        <v>58</v>
+      </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.4">
+    <row r="37" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B37" s="5">
         <v>200</v>
       </c>
@@ -10893,6 +12953,9 @@
       </c>
       <c r="D37" s="5" t="str">
         <v>{"gamma_gas":0.6,"gamma_oil":0.86,"gamma_wat":1,"rsb_m3m3":69.495,"pb_atma":155.315,"t_res_C":90,"bob_m3m3":1.225,"muob_cP":0.738,"PVT_corr_set":0,"q_liq_sm3day":200,"fw_perc":0,"rp_m3m3":69.495}</v>
+      </c>
+      <c r="E37" t="s">
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>